<commit_message>
Added the face validation tc
</commit_message>
<xml_diff>
--- a/excel/Proctoring Pro.xlsx
+++ b/excel/Proctoring Pro.xlsx
@@ -529,23 +529,21 @@
       </c>
       <c r="G2" s="15" t="inlineStr">
         <is>
-          <t>NOT EXECUTED in Cowork sandbox.
-Test artifacts generated &amp; validated (node require/syntax checks pass for all 5):
-  - pages/StudentLMSPage.js (locators only)
-  - actions/StudentLMSActions.js (loginAsStudent, openCourseQuiz, clickAttemptOrContinue, clickValidateFace, verifyFaceValidationMatched)
-  - tests/regression/studentTests.spec.js (TC-1 spec, uses customfixture)
-  - tests/fixture/customfixture.js (registers actions.studentLms; safeRequire'd missing OrangeHRM actions)
-  - config/env.config.js + .env.example (LMS_BASE_URL, LMS_STUDENT_EMAIL, LMS_STUDENT_PASSWORD, LMS_COURSE_NAME)
-Why execution was skipped here:
-  1) Chromium install blocked: 'npx playwright install chromium' fails (sudo disabled + download endpoint unreachable in this sandbox).
-  2) Target host education.elearning23.com is NOT on the Cowork egress allowlist; even an HTTP probe is rejected.
-  3) Real face validation needs a webcam; sandbox has no video device. Locally use --use-fake-device-for-media-stream with --use-file-for-fake-video-capture pointing at the baseline-face image.
-Run locally to capture the real Actual Result:
-  1) cp .env.example .env  -- set LMS_STUDENT_EMAIL / LMS_STUDENT_PASSWORD
-  2) npm install
-  3) npx playwright install chromium
-  4) npx playwright test tests/regression/studentTests.spec.js --headed
-  5) Paste the run summary back; this cell will be overwritten with the real PASS/FAIL outcome.</t>
+          <t>[2026-05-07_07-41-32] NOT EXECUTED in Cowork sandbox.
+Blockers (verified just now):
+  1. `npx playwright install chromium` -&gt; 403 "Connection blocked by network allowlist"
+     (https://playwright.azureedge.net/builds/chromium/1148/...)
+  2. https://education.elearning23.com/ -&gt; HTTP 000 (host not on egress allowlist)
+  3. /dev/video* absent (irrelevant once fake-media flags are on, but noted)
+Code is ready. To run locally:
+  1. Drop the real student photo at data/fixtures/face/baseline.jpg (640x480 JPEG)
+  2. bash data/fixtures/face/generate-y4m.sh
+  3. cp .env.example .env  -- set LMS_STUDENT_EMAIL / LMS_STUDENT_PASSWORD
+  4. npm install &amp;&amp; npx playwright install chromium
+  5. npx playwright test tests/regression/                    -- runs all 5 specs / 7 tests
+     # or one spec at a time:
+     npx playwright test tests/regression/studentTests.spec.js --headed
+ExcelResultWriter will overwrite this cell with the real PASS/FAIL on each run.</t>
         </is>
       </c>
       <c r="H2" s="10" t="inlineStr">
@@ -574,14 +572,67 @@
       <c r="AA2" s="6" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="n"/>
-      <c r="B3" s="10" t="n"/>
-      <c r="C3" s="12" t="n"/>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
+      <c r="A3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Face mismatch on quiz start</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Go to https://education.elearning23.com/
+Login as student:
+  sazidnx23@yopmail.com / Admin@123
+Open course "Computational Problem Solving" → quiz
+Camera: Chromium fake-media flags fed via Y4M file from data/fixtures/face/.
+See data/fixtures/face/README.md for replacing baseline.jpg with the real student photo.
+This TC overrides launchOptions to feed mismatch.y4m as the camera stream.</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Stored photo is the student; live camera feed is a different person — face validation must REJECT.</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>1. Open quiz
+2. Click the Attempt Quiz / Continue Attempt button
+3. Click Validate Face button
+   (Camera feed = data/fixtures/face/mismatch.y4m)</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>Popup shows "Face Validation: Face not matched." (or equivalent rejection message). Validate Face button does NOT advance to Start Attempt.</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>[2026-05-07_07-41-32] NOT EXECUTED in Cowork sandbox.
+Blockers (verified just now):
+  1. `npx playwright install chromium` -&gt; 403 "Connection blocked by network allowlist"
+     (https://playwright.azureedge.net/builds/chromium/1148/...)
+  2. https://education.elearning23.com/ -&gt; HTTP 000 (host not on egress allowlist)
+  3. /dev/video* absent (irrelevant once fake-media flags are on, but noted)
+Code is ready. To run locally:
+  1. Drop the real student photo at data/fixtures/face/baseline.jpg (640x480 JPEG)
+  2. bash data/fixtures/face/generate-y4m.sh
+  3. cp .env.example .env  -- set LMS_STUDENT_EMAIL / LMS_STUDENT_PASSWORD
+  4. npm install &amp;&amp; npx playwright install chromium
+  5. npx playwright test tests/regression/                    -- runs all 5 specs / 7 tests
+     # or one spec at a time:
+     npx playwright test tests/regression/studentTests.spec.js --headed
+ExcelResultWriter will overwrite this cell with the real PASS/FAIL on each run.</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>Negative test for face match. Mismatch fixture is synthetic on purpose.</t>
+        </is>
+      </c>
       <c r="I3" s="10" t="n"/>
       <c r="J3" s="10" t="n"/>
       <c r="K3" s="6" t="n"/>
@@ -603,14 +654,66 @@
       <c r="AA3" s="6" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="n"/>
-      <c r="B4" s="10" t="n"/>
-      <c r="C4" s="12" t="n"/>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="10" t="n"/>
-      <c r="F4" s="10" t="n"/>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="10" t="n"/>
+      <c r="A4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Camera permission denied</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Go to https://education.elearning23.com/
+Login as student:
+  sazidnx23@yopmail.com / Admin@123
+Open course "Computational Problem Solving" → quiz
+Camera: Chromium fake-media flags fed via Y4M file from data/fixtures/face/.
+See data/fixtures/face/README.md for replacing baseline.jpg with the real student photo.
+This TC clears camera permissions before the quiz opens, simulating the user clicking Block in the browser permission prompt.</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>When the student denies camera access, Proctoring Pro must surface a camera-permission error instead of silently failing.</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>1. Open quiz with camera permission BLOCKED
+2. Click the Attempt Quiz / Continue Attempt button
+3. Click Validate Face button</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>A camera-permission / "Allow camera access" error message is visible. The student cannot proceed to Start Attempt.</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>[2026-05-07_07-41-32] NOT EXECUTED in Cowork sandbox.
+Blockers (verified just now):
+  1. `npx playwright install chromium` -&gt; 403 "Connection blocked by network allowlist"
+     (https://playwright.azureedge.net/builds/chromium/1148/...)
+  2. https://education.elearning23.com/ -&gt; HTTP 000 (host not on egress allowlist)
+  3. /dev/video* absent (irrelevant once fake-media flags are on, but noted)
+Code is ready. To run locally:
+  1. Drop the real student photo at data/fixtures/face/baseline.jpg (640x480 JPEG)
+  2. bash data/fixtures/face/generate-y4m.sh
+  3. cp .env.example .env  -- set LMS_STUDENT_EMAIL / LMS_STUDENT_PASSWORD
+  4. npm install &amp;&amp; npx playwright install chromium
+  5. npx playwright test tests/regression/                    -- runs all 5 specs / 7 tests
+     # or one spec at a time:
+     npx playwright test tests/regression/studentTests.spec.js --headed
+ExcelResultWriter will overwrite this cell with the real PASS/FAIL on each run.</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Verifies graceful handling of denied permissions.</t>
+        </is>
+      </c>
       <c r="I4" s="10" t="n"/>
       <c r="J4" s="10" t="n"/>
       <c r="K4" s="6" t="n"/>
@@ -632,14 +735,66 @@
       <c r="AA4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n"/>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="12" t="n"/>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="10" t="n"/>
+      <c r="A5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>No camera device available</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Go to https://education.elearning23.com/
+Login as student:
+  sazidnx23@yopmail.com / Admin@123
+Open course "Computational Problem Solving" → quiz
+Camera: Chromium fake-media flags fed via Y4M file from data/fixtures/face/.
+See data/fixtures/face/README.md for replacing baseline.jpg with the real student photo.
+Launched WITHOUT --use-fake-device-for-media-stream so Chromium reports no video device.</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>When no webcam is attached, the plugin must show a "no camera detected" message rather than crash.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>1. Open quiz on a machine with no webcam (or Chromium launched without fake-media flags)
+2. Click the Attempt Quiz / Continue Attempt button
+3. Click Validate Face button</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>A "No camera detected" or equivalent error is shown. The Validate Face flow does not proceed.</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>[2026-05-07_07-41-32] NOT EXECUTED in Cowork sandbox.
+Blockers (verified just now):
+  1. `npx playwright install chromium` -&gt; 403 "Connection blocked by network allowlist"
+     (https://playwright.azureedge.net/builds/chromium/1148/...)
+  2. https://education.elearning23.com/ -&gt; HTTP 000 (host not on egress allowlist)
+  3. /dev/video* absent (irrelevant once fake-media flags are on, but noted)
+Code is ready. To run locally:
+  1. Drop the real student photo at data/fixtures/face/baseline.jpg (640x480 JPEG)
+  2. bash data/fixtures/face/generate-y4m.sh
+  3. cp .env.example .env  -- set LMS_STUDENT_EMAIL / LMS_STUDENT_PASSWORD
+  4. npm install &amp;&amp; npx playwright install chromium
+  5. npx playwright test tests/regression/                    -- runs all 5 specs / 7 tests
+     # or one spec at a time:
+     npx playwright test tests/regression/studentTests.spec.js --headed
+ExcelResultWriter will overwrite this cell with the real PASS/FAIL on each run.</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>Hardware-availability negative path.</t>
+        </is>
+      </c>
       <c r="I5" s="10" t="n"/>
       <c r="J5" s="10" t="n"/>
       <c r="K5" s="6" t="n"/>
@@ -661,14 +816,68 @@
       <c r="AA5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="n"/>
-      <c r="B6" s="10" t="n"/>
-      <c r="C6" s="12" t="n"/>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
-      <c r="H6" s="10" t="n"/>
+      <c r="A6" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Suspicious activity — no face / multiple faces</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Go to https://education.elearning23.com/
+Login as student:
+  sazidnx23@yopmail.com / Admin@123
+Open course "Computational Problem Solving" → quiz
+Camera: Chromium fake-media flags fed via Y4M file from data/fixtures/face/.
+See data/fixtures/face/README.md for replacing baseline.jpg with the real student photo.
+Leg A camera feed = no-face.y4m (empty room). Leg B camera feed = multi-face.y4m (two people).</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Proctoring Pro must flag suspicious frames: empty room (no face) and multiple faces simultaneously.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>1. Open quiz with no-face camera feed
+2. Click Attempt / Continue Attempt
+3. Click Validate Face
+4. Repeat with multi-face feed</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>Leg A: "No face detected" warning is visible.
+Leg B: "Multiple faces detected" warning OR a suspicious-activity banner is visible.</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>[2026-05-07_07-41-32] NOT EXECUTED in Cowork sandbox.
+Blockers (verified just now):
+  1. `npx playwright install chromium` -&gt; 403 "Connection blocked by network allowlist"
+     (https://playwright.azureedge.net/builds/chromium/1148/...)
+  2. https://education.elearning23.com/ -&gt; HTTP 000 (host not on egress allowlist)
+  3. /dev/video* absent (irrelevant once fake-media flags are on, but noted)
+Code is ready. To run locally:
+  1. Drop the real student photo at data/fixtures/face/baseline.jpg (640x480 JPEG)
+  2. bash data/fixtures/face/generate-y4m.sh
+  3. cp .env.example .env  -- set LMS_STUDENT_EMAIL / LMS_STUDENT_PASSWORD
+  4. npm install &amp;&amp; npx playwright install chromium
+  5. npx playwright test tests/regression/                    -- runs all 5 specs / 7 tests
+     # or one spec at a time:
+     npx playwright test tests/regression/studentTests.spec.js --headed
+ExcelResultWriter will overwrite this cell with the real PASS/FAIL on each run.</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>Both legs run under TC-5; either failure fails the row.</t>
+        </is>
+      </c>
       <c r="I6" s="10" t="n"/>
       <c r="J6" s="10" t="n"/>
       <c r="K6" s="6" t="n"/>
@@ -690,14 +899,69 @@
       <c r="AA6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="13" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
+      <c r="A7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Full proctoring flow (match → start → submit)</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Go to https://education.elearning23.com/
+Login as student:
+  sazidnx23@yopmail.com / Admin@123
+Open course "Computational Problem Solving" → quiz
+Camera: Chromium fake-media flags fed via Y4M file from data/fixtures/face/.
+See data/fixtures/face/README.md for replacing baseline.jpg with the real student photo.
+Default baseline.y4m camera feed — face will match.</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Happy-path E2E: face matches, student starts the attempt, the webcam preview stays visible during the quiz, and the attempt is submitted.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>1. Open quiz
+2. Click Attempt / Continue Attempt
+3. Click Validate Face → "Face matched"
+4. Click Start Attempt
+5. Verify the webcam preview tile + first quiz question are visible
+6. Click Finish Attempt → Submit All and Finish</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Quiz transitions through validation → attempt → review/summary without errors. Webcam preview remains visible while the quiz is open.</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>[2026-05-07_07-41-32] NOT EXECUTED in Cowork sandbox.
+Blockers (verified just now):
+  1. `npx playwright install chromium` -&gt; 403 "Connection blocked by network allowlist"
+     (https://playwright.azureedge.net/builds/chromium/1148/...)
+  2. https://education.elearning23.com/ -&gt; HTTP 000 (host not on egress allowlist)
+  3. /dev/video* absent (irrelevant once fake-media flags are on, but noted)
+Code is ready. To run locally:
+  1. Drop the real student photo at data/fixtures/face/baseline.jpg (640x480 JPEG)
+  2. bash data/fixtures/face/generate-y4m.sh
+  3. cp .env.example .env  -- set LMS_STUDENT_EMAIL / LMS_STUDENT_PASSWORD
+  4. npm install &amp;&amp; npx playwright install chromium
+  5. npx playwright test tests/regression/                    -- runs all 5 specs / 7 tests
+     # or one spec at a time:
+     npx playwright test tests/regression/studentTests.spec.js --headed
+ExcelResultWriter will overwrite this cell with the real PASS/FAIL on each run.</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Smoke E2E for the full proctoring journey.</t>
+        </is>
+      </c>
       <c r="I7" s="6" t="n"/>
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>

</xml_diff>

<commit_message>
add the testcase and update the skill
</commit_message>
<xml_diff>
--- a/excel/Proctoring Pro.xlsx
+++ b/excel/Proctoring Pro.xlsx
@@ -8,19 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bs01383/Documents/playreltemp/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAFB089C-CB33-6D41-9DBB-00B9FC097686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{297E5F61-1DBE-4C4A-9204-C5620EA4AAEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-3580" yWindow="-21000" windowWidth="38400" windowHeight="21000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Student" sheetId="1" r:id="rId1"/>
+    <sheet name="Admin" sheetId="2" r:id="rId2"/>
+    <sheet name="Teacher" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="62">
   <si>
     <t>ID</t>
   </si>
@@ -67,23 +69,6 @@
   </si>
   <si>
     <t>Face validation only show like  "Face Validation: Face matched." in the popup</t>
-  </si>
-  <si>
-    <t>[2026-05-07_07-41-32] NOT EXECUTED in Cowork sandbox.
-Blockers (verified just now):
-  1. `npx playwright install chromium` -&gt; 403 "Connection blocked by network allowlist"
-     (https://playwright.azureedge.net/builds/chromium/1148/...)
-  2. https://education.elearning23.com/ -&gt; HTTP 000 (host not on egress allowlist)
-  3. /dev/video* absent (irrelevant once fake-media flags are on, but noted)
-Code is ready. To run locally:
-  1. Drop the real student photo at data/fixtures/face/baseline.jpg (640x480 JPEG)
-  2. bash data/fixtures/face/generate-y4m.sh
-  3. cp .env.example .env  -- set LMS_STUDENT_EMAIL / LMS_STUDENT_PASSWORD
-  4. npm install &amp;&amp; npx playwright install chromium
-  5. npx playwright test tests/regression/                    -- runs all 5 specs / 7 tests
-     # or one spec at a time:
-     npx playwright test tests/regression/studentTests.spec.js --headed
-ExcelResultWriter will overwrite this cell with the real PASS/FAIL on each run.</t>
   </si>
   <si>
     <t>Verifies identity</t>
@@ -244,12 +229,60 @@
   <si>
     <t>User will see the homepage after logout. Here is the homepage url: https://education.elearning23.com/</t>
   </si>
+  <si>
+    <t>Log in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Go to https://education.elearning23.com/
+Login as admin:
+  sazid_admin / Punch@500#$
+</t>
+  </si>
+  <si>
+    <t>Admin can login and see the deashboard</t>
+  </si>
+  <si>
+    <t>1. Login as admin
+2. See the Dashboard Keyword</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The admin sees the dashboard after login. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Go to https://education.elearning23.com/
+Login as teacher:
+  teacher / Admin@123
+</t>
+  </si>
+  <si>
+    <t>Teacher can login and see the deashboard</t>
+  </si>
+  <si>
+    <t>1. Login as Teacher
+2. See the Dashboard Keyword</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The teacher sees the dashboard after login. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Go to https://education.elearning23.com/
+</t>
+  </si>
+  <si>
+    <t>Admin can Logout from the system in the course</t>
+  </si>
+  <si>
+    <t>Teacher can Logout from the system in the course</t>
+  </si>
+  <si>
+    <t>Teacher will see the homepage after logout. Here is the homepage url: https://education.elearning23.com/</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -294,13 +327,8 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -313,13 +341,8 @@
         <bgColor rgb="FF0A2F41"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -342,11 +365,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -371,9 +409,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -381,6 +416,29 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -607,8 +665,8 @@
     <col min="2" max="2" width="42.83203125" customWidth="1"/>
     <col min="3" max="3" width="31.6640625" customWidth="1"/>
     <col min="4" max="4" width="49.33203125" customWidth="1"/>
-    <col min="5" max="5" width="50.33203125" style="14" customWidth="1"/>
-    <col min="6" max="6" width="67.83203125" style="14" customWidth="1"/>
+    <col min="5" max="5" width="50.33203125" style="13" customWidth="1"/>
+    <col min="6" max="6" width="67.83203125" style="13" customWidth="1"/>
     <col min="7" max="7" width="70" customWidth="1"/>
     <col min="8" max="8" width="58.6640625" customWidth="1"/>
   </cols>
@@ -629,7 +687,7 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="14" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
@@ -671,17 +729,15 @@
       <c r="D2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="12" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="6"/>
+      <c r="H2" s="5" t="s">
         <v>13</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>14</v>
       </c>
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
@@ -703,30 +759,28 @@
       <c r="Z2" s="6"/>
       <c r="AA2" s="6"/>
     </row>
-    <row r="3" spans="1:27" ht="266">
+    <row r="3" spans="1:27" ht="240">
       <c r="A3" s="7">
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="F3" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="6"/>
+      <c r="H3" s="5" t="s">
         <v>19</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>20</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
@@ -748,30 +802,28 @@
       <c r="Z3" s="6"/>
       <c r="AA3" s="6"/>
     </row>
-    <row r="4" spans="1:27" ht="266">
+    <row r="4" spans="1:27" ht="255">
       <c r="A4" s="7">
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="F4" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="G4" s="6"/>
+      <c r="H4" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
@@ -793,30 +845,28 @@
       <c r="Z4" s="6"/>
       <c r="AA4" s="6"/>
     </row>
-    <row r="5" spans="1:27" ht="266">
+    <row r="5" spans="1:27" ht="240">
       <c r="A5" s="7">
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="D5" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="F5" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="G5" s="6"/>
+      <c r="H5" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
@@ -838,30 +888,28 @@
       <c r="Z5" s="6"/>
       <c r="AA5" s="6"/>
     </row>
-    <row r="6" spans="1:27" ht="266">
+    <row r="6" spans="1:27" ht="240">
       <c r="A6" s="7">
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="D6" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="F6" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="G6" s="6"/>
+      <c r="H6" s="5" t="s">
         <v>37</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>38</v>
       </c>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
@@ -883,30 +931,28 @@
       <c r="Z6" s="6"/>
       <c r="AA6" s="6"/>
     </row>
-    <row r="7" spans="1:27" ht="266">
+    <row r="7" spans="1:27" ht="225">
       <c r="A7" s="7">
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="D7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="F7" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="G7" s="6"/>
+      <c r="H7" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>44</v>
       </c>
       <c r="I7" s="6"/>
       <c r="J7" s="6"/>
@@ -933,19 +979,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="D8" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="F8" s="11" t="s">
         <v>48</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>49</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
@@ -29714,4 +29760,298 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C9670BE-61C2-F448-82E5-A4CFED97EBF5}">
+  <dimension ref="A1:AA3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
+  <cols>
+    <col min="1" max="1" width="26.83203125" style="22" customWidth="1"/>
+    <col min="2" max="2" width="31.5" style="22" customWidth="1"/>
+    <col min="3" max="3" width="33.6640625" style="22" customWidth="1"/>
+    <col min="4" max="4" width="67.33203125" style="22" customWidth="1"/>
+    <col min="5" max="5" width="43.5" style="22" customWidth="1"/>
+    <col min="6" max="6" width="34.83203125" style="22" customWidth="1"/>
+    <col min="7" max="7" width="31.33203125" style="22" customWidth="1"/>
+    <col min="8" max="16384" width="10.83203125" style="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:27" ht="17">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
+      <c r="Q1" s="21"/>
+      <c r="R1" s="21"/>
+      <c r="S1" s="21"/>
+      <c r="T1" s="21"/>
+      <c r="U1" s="21"/>
+      <c r="V1" s="21"/>
+      <c r="W1" s="21"/>
+      <c r="X1" s="21"/>
+      <c r="Y1" s="21"/>
+      <c r="Z1" s="21"/>
+      <c r="AA1" s="21"/>
+    </row>
+    <row r="2" spans="1:27" ht="90">
+      <c r="A2" s="21">
+        <v>1</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
+      <c r="M2" s="21"/>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21"/>
+      <c r="P2" s="21"/>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="S2" s="21"/>
+      <c r="T2" s="21"/>
+      <c r="U2" s="21"/>
+      <c r="V2" s="21"/>
+      <c r="W2" s="21"/>
+      <c r="X2" s="21"/>
+      <c r="Y2" s="21"/>
+      <c r="Z2" s="21"/>
+      <c r="AA2" s="21"/>
+    </row>
+    <row r="3" spans="1:27" customFormat="1" ht="45">
+      <c r="A3" s="6">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B659DA00-9B82-2D46-9CEE-F5E4770E1EAE}">
+  <dimension ref="A1:AA3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
+  <cols>
+    <col min="1" max="1" width="26.83203125" style="22" customWidth="1"/>
+    <col min="2" max="2" width="31.5" style="22" customWidth="1"/>
+    <col min="3" max="3" width="33.6640625" style="22" customWidth="1"/>
+    <col min="4" max="4" width="67.33203125" style="22" customWidth="1"/>
+    <col min="5" max="5" width="43.5" style="22" customWidth="1"/>
+    <col min="6" max="6" width="34.83203125" style="22" customWidth="1"/>
+    <col min="7" max="7" width="31.33203125" style="22" customWidth="1"/>
+    <col min="8" max="16384" width="10.83203125" style="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:27" ht="17">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
+      <c r="Q1" s="21"/>
+      <c r="R1" s="21"/>
+      <c r="S1" s="21"/>
+      <c r="T1" s="21"/>
+      <c r="U1" s="21"/>
+      <c r="V1" s="21"/>
+      <c r="W1" s="21"/>
+      <c r="X1" s="21"/>
+      <c r="Y1" s="21"/>
+      <c r="Z1" s="21"/>
+      <c r="AA1" s="21"/>
+    </row>
+    <row r="2" spans="1:27" ht="90">
+      <c r="A2" s="21">
+        <v>1</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="E2" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
+      <c r="K2" s="21"/>
+      <c r="L2" s="21"/>
+      <c r="M2" s="21"/>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21"/>
+      <c r="P2" s="21"/>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="S2" s="21"/>
+      <c r="T2" s="21"/>
+      <c r="U2" s="21"/>
+      <c r="V2" s="21"/>
+      <c r="W2" s="21"/>
+      <c r="X2" s="21"/>
+      <c r="Y2" s="21"/>
+      <c r="Z2" s="21"/>
+      <c r="AA2" s="21"/>
+    </row>
+    <row r="3" spans="1:27" customFormat="1" ht="45">
+      <c r="A3" s="6">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>